<commit_message>
Add STOTEN revision analyses: alternative baselines, uncertainty, emission-weighted CAGR
Adds three new sensitivity/robustness scripts (alternative baseline years,
inventory uncertainty propagation, emission-weighted CAGR), drops the
SDG 13.2 status labels from outputs in favor of plain trajectory names,
and updates the README and .gitignore allowlist to track the new output
tables and figures.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GHG_Trajectory_Analysis_Study/outputs/tables/Sensitivity Analysis_Threshold.xlsx
+++ b/GHG_Trajectory_Analysis_Study/outputs/tables/Sensitivity Analysis_Threshold.xlsx
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,21 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,59 +419,59 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>System</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Stable threshold</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Mod. Rising threshold</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Rapid Rising threshold</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>N Declining</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>N Stable</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>N Mod. Rising</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>N Rapidly Rising</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Countries reclassified</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Reclassified (%)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Headline holds (&gt;50% SDG 13.2-Critical)</t>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Headline holds (&gt;50% Rapidly Rising)</t>
         </is>
       </c>
     </row>
@@ -643,27 +631,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>GHG Change 1970-2024 (%)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Baseline Class</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Set A Class</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Reclassification</t>
         </is>
@@ -934,27 +922,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>GHG Change 1970-2024 (%)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Baseline Class</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Set B Class</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Reclassification</t>
         </is>

</xml_diff>